<commit_message>
Troca logotipo para Aprosoja I + corrige campo Área no PWA + feedback formulário
</commit_message>
<xml_diff>
--- a/Dados_Produtores.xlsx
+++ b/Dados_Produtores.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="4" activeTab="9" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUÇÕES" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,8 +16,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anaurilândia (Soja)" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Antônio João (Soja)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aparecida do Taboado (Soja)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rio Brilhante (Soja)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Angélica (Soja)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -27,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,27 +63,16 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1B4332"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -115,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,9 +116,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -552,39 +536,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="10.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="7.88671875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="20.21875" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="19.88671875" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="18.44140625" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="13.5546875" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="26.21875" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="20" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="14.88671875" bestFit="1" customWidth="1" min="10" max="10"/>
-    <col width="13.21875" bestFit="1" customWidth="1" min="11" max="12"/>
-    <col width="13.33203125" bestFit="1" customWidth="1" min="13" max="13"/>
-    <col width="15" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="13.88671875" bestFit="1" customWidth="1" min="15" max="15"/>
-    <col width="19.109375" bestFit="1" customWidth="1" min="16" max="16"/>
-    <col width="18.44140625" bestFit="1" customWidth="1" min="17" max="17"/>
-    <col width="21.6640625" bestFit="1" customWidth="1" min="18" max="18"/>
-    <col width="17.44140625" bestFit="1" customWidth="1" min="19" max="19"/>
-    <col width="21.6640625" bestFit="1" customWidth="1" min="20" max="20"/>
-    <col width="25.109375" bestFit="1" customWidth="1" min="21" max="21"/>
-    <col width="16.109375" bestFit="1" customWidth="1" min="22" max="22"/>
-    <col width="24" bestFit="1" customWidth="1" min="23" max="23"/>
-    <col width="24.109375" bestFit="1" customWidth="1" min="24" max="24"/>
-    <col width="15.5546875" bestFit="1" customWidth="1" min="25" max="25"/>
-    <col width="17.109375" bestFit="1" customWidth="1" min="26" max="26"/>
-    <col width="16.77734375" bestFit="1" customWidth="1" min="27" max="27"/>
-    <col width="13.77734375" bestFit="1" customWidth="1" min="28" max="28"/>
-    <col width="13.33203125" bestFit="1" customWidth="1" min="29" max="29"/>
-    <col width="15" bestFit="1" customWidth="1" min="30" max="30"/>
-    <col width="16.21875" bestFit="1" customWidth="1" min="31" max="31"/>
-    <col width="27.109375" bestFit="1" customWidth="1" min="32" max="32"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
@@ -850,566 +802,6 @@
       </c>
       <c r="AF2" t="n">
         <v>2.708333333333333</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Técnico</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Município</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>Área (ha)</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>Produtividade (sc/ha)</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>Preço Venda (R$/sc)</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Sementes (R$)</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>Tratamento de Semente (R$)</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>Corretivo de Solo (R$)</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>Fertilizante (R$)</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>Fungicida (R$)</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>Herbicida (R$)</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>Inseticida (R$)</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>Inoculantes (R$)</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>Adjuvante (R$)</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>Op. c/ Máquinas (R$)</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>Seguro Agrícola (R$)</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>Transporte Externo (R$)</t>
-        </is>
-      </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>Armazenagem (R$)</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>Assistência Técnica (R$)</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
-        <is>
-          <t>Manutenção Máquinas (R$)</t>
-        </is>
-      </c>
-      <c r="V1" s="7" t="inlineStr">
-        <is>
-          <t>Mão de Obra (R$)</t>
-        </is>
-      </c>
-      <c r="W1" s="7" t="inlineStr">
-        <is>
-          <t>Desp. Administrativas (R$)</t>
-        </is>
-      </c>
-      <c r="X1" s="7" t="inlineStr">
-        <is>
-          <t>Juros/Financiamentos (R$)</t>
-        </is>
-      </c>
-      <c r="Y1" s="7" t="inlineStr">
-        <is>
-          <t>Depreciação (R$)</t>
-        </is>
-      </c>
-      <c r="Z1" s="7" t="inlineStr">
-        <is>
-          <t>Outros Custos (R$)</t>
-        </is>
-      </c>
-      <c r="AA1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL (R$)</t>
-        </is>
-      </c>
-      <c r="AB1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AC1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO/sc (R$)</t>
-        </is>
-      </c>
-      <c r="AD1" s="7" t="inlineStr">
-        <is>
-          <t>RECEITA/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AE1" s="7" t="inlineStr">
-        <is>
-          <t>MARGEM/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AF1" s="7" t="inlineStr">
-        <is>
-          <t>PONTO DE EQUILÍBRIO (sc/ha)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Linneu</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Rio Brilhante</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>45</v>
-      </c>
-      <c r="E2" t="n">
-        <v>62</v>
-      </c>
-      <c r="F2" t="n">
-        <v>120</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>14625</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>14625</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>325</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>5.241935483870968</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>7440</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>7115</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>2.708333333333333</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Técnico</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Município</t>
-        </is>
-      </c>
-      <c r="D1" s="7" t="inlineStr">
-        <is>
-          <t>Área (ha)</t>
-        </is>
-      </c>
-      <c r="E1" s="7" t="inlineStr">
-        <is>
-          <t>Produtividade (sc/ha)</t>
-        </is>
-      </c>
-      <c r="F1" s="7" t="inlineStr">
-        <is>
-          <t>Preço Venda (R$/sc)</t>
-        </is>
-      </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Sementes (R$)</t>
-        </is>
-      </c>
-      <c r="H1" s="7" t="inlineStr">
-        <is>
-          <t>Tratamento de Semente (R$)</t>
-        </is>
-      </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>Corretivo de Solo (R$)</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>Fertilizante (R$)</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>Fungicida (R$)</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>Herbicida (R$)</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>Inseticida (R$)</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>Inoculantes (R$)</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>Adjuvante (R$)</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>Op. c/ Máquinas (R$)</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>Seguro Agrícola (R$)</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>Transporte Externo (R$)</t>
-        </is>
-      </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>Armazenagem (R$)</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>Assistência Técnica (R$)</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
-        <is>
-          <t>Manutenção Máquinas (R$)</t>
-        </is>
-      </c>
-      <c r="V1" s="7" t="inlineStr">
-        <is>
-          <t>Mão de Obra (R$)</t>
-        </is>
-      </c>
-      <c r="W1" s="7" t="inlineStr">
-        <is>
-          <t>Desp. Administrativas (R$)</t>
-        </is>
-      </c>
-      <c r="X1" s="7" t="inlineStr">
-        <is>
-          <t>Juros/Financiamentos (R$)</t>
-        </is>
-      </c>
-      <c r="Y1" s="7" t="inlineStr">
-        <is>
-          <t>Depreciação (R$)</t>
-        </is>
-      </c>
-      <c r="Z1" s="7" t="inlineStr">
-        <is>
-          <t>Outros Custos (R$)</t>
-        </is>
-      </c>
-      <c r="AA1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO TOTAL (R$)</t>
-        </is>
-      </c>
-      <c r="AB1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AC1" s="7" t="inlineStr">
-        <is>
-          <t>CUSTO/sc (R$)</t>
-        </is>
-      </c>
-      <c r="AD1" s="7" t="inlineStr">
-        <is>
-          <t>RECEITA/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AE1" s="7" t="inlineStr">
-        <is>
-          <t>MARGEM/ha (R$)</t>
-        </is>
-      </c>
-      <c r="AF1" s="7" t="inlineStr">
-        <is>
-          <t>PONTO DE EQUILÍBRIO (sc/ha)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-06-02</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Raphael</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Angélica</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>60</v>
-      </c>
-      <c r="E2" t="n">
-        <v>60</v>
-      </c>
-      <c r="F2" t="n">
-        <v>120</v>
-      </c>
-      <c r="G2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H2" t="n">
-        <v>6464</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>19500</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>31964</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>532.7333333333333</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>8.878888888888889</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>7200</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>6667.266666666666</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>4.439444444444445</v>
       </c>
     </row>
   </sheetData>
@@ -2740,7 +2132,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3020,7 +2412,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
@@ -3300,7 +2692,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AF2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="inlineStr">

</xml_diff>